<commit_message>
- Fix pregnancy_visit_ext.xlsx HForm syntax error. - Update main gsp copypright
</commit_message>
<xml_diff>
--- a/src/main/resources/samples/extension-forms/xls-hforms/pregnancy_visit_ext.xlsx
+++ b/src/main/resources/samples/extension-forms/xls-hforms/pregnancy_visit_ext.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3065" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3065" uniqueCount="146">
   <si>
     <t>group</t>
   </si>
@@ -106,9 +106,6 @@
   </si>
   <si>
     <t>Código da Mãe</t>
-  </si>
-  <si>
-    <t>trur</t>
   </si>
   <si>
     <t>mother_name</t>
@@ -464,10 +461,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -483,10 +480,25 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -497,8 +509,107 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -514,123 +625,9 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -661,13 +658,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -679,43 +682,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -727,7 +694,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -745,7 +712,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -757,7 +766,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -769,13 +814,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -787,55 +826,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -849,11 +846,62 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -878,47 +926,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -931,168 +943,153 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1653,7 +1650,7 @@
         <v>23</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="O4" s="8" t="s">
         <v>18</v>
@@ -1673,7 +1670,7 @@
         <v>18</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>20</v>
@@ -1682,10 +1679,10 @@
         <v>18</v>
       </c>
       <c r="G5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>32</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>33</v>
       </c>
       <c r="I5" s="8" t="s">
         <v>18</v>
@@ -1723,22 +1720,22 @@
         <v>18</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="E6" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="F6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="9" t="s">
+      <c r="H6" s="9" t="s">
         <v>37</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>38</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>18</v>
@@ -1776,19 +1773,19 @@
         <v>18</v>
       </c>
       <c r="C7" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="F7" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="9" t="s">
+      <c r="H7" s="9" t="s">
         <v>41</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>42</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>18</v>
@@ -1826,22 +1823,22 @@
         <v>18</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F8" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="9" t="s">
+      <c r="H8" s="9" t="s">
         <v>45</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>46</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>18</v>
@@ -1879,19 +1876,19 @@
         <v>18</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="9" t="s">
+      <c r="H9" s="9" t="s">
         <v>48</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>49</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>18</v>
@@ -1929,19 +1926,19 @@
         <v>18</v>
       </c>
       <c r="C10" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="H10" s="7" t="s">
         <v>53</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>54</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>18</v>
@@ -1979,22 +1976,22 @@
         <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>18</v>
@@ -2032,7 +2029,7 @@
         <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>20</v>
@@ -2041,10 +2038,10 @@
         <v>18</v>
       </c>
       <c r="G12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>18</v>
@@ -2082,7 +2079,7 @@
         <v>18</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>20</v>
@@ -2091,10 +2088,10 @@
         <v>18</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>18</v>
@@ -2132,22 +2129,22 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>18</v>
@@ -2185,22 +2182,22 @@
         <v>18</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>18</v>
@@ -2238,7 +2235,7 @@
         <v>18</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>20</v>
@@ -2247,10 +2244,10 @@
         <v>18</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>18</v>
@@ -2288,7 +2285,7 @@
         <v>18</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>20</v>
@@ -2297,10 +2294,10 @@
         <v>18</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>18</v>
@@ -2338,10 +2335,10 @@
         <v>18</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>18</v>
@@ -2385,7 +2382,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>20</v>
@@ -2394,10 +2391,10 @@
         <v>18</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>18</v>
@@ -2435,7 +2432,7 @@
         <v>18</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>20</v>
@@ -2444,10 +2441,10 @@
         <v>18</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>18</v>
@@ -2508,13 +2505,13 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>13</v>
@@ -2528,16 +2525,16 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>18</v>
@@ -2551,16 +2548,16 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>89</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>18</v>
@@ -2574,16 +2571,16 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>18</v>
@@ -2597,16 +2594,16 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>18</v>
@@ -2620,16 +2617,16 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>18</v>
@@ -2643,16 +2640,16 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>18</v>
@@ -2666,16 +2663,16 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>106</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>18</v>
@@ -2689,16 +2686,16 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>18</v>
@@ -2712,16 +2709,16 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>18</v>
@@ -2735,16 +2732,16 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>18</v>
@@ -2758,16 +2755,16 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>18</v>
@@ -2781,16 +2778,16 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>18</v>
@@ -2804,16 +2801,16 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>18</v>
@@ -2827,16 +2824,16 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>18</v>
@@ -2850,16 +2847,16 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>18</v>
@@ -2873,16 +2870,16 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>18</v>
@@ -2896,16 +2893,16 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>18</v>
@@ -2919,16 +2916,16 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>18</v>
@@ -2942,16 +2939,16 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>18</v>
@@ -2965,16 +2962,16 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>18</v>
@@ -11494,30 +11491,30 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>145</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>146</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
- Update hform pregnancy_visit_ext.xlsx - Add TIMESTAMP to DatabaseColumnType and FormColumnType - Fix copy of collected_id on some services - Add missing id column on household_proxy_head extension table
</commit_message>
<xml_diff>
--- a/src/main/resources/samples/extension-forms/xls-hforms/pregnancy_visit_ext.xlsx
+++ b/src/main/resources/samples/extension-forms/xls-hforms/pregnancy_visit_ext.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3065" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3064" uniqueCount="146">
   <si>
     <t>group</t>
   </si>
@@ -461,10 +461,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -496,74 +496,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -577,8 +510,47 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -594,17 +566,30 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -616,11 +601,26 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -658,31 +658,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -694,7 +694,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -712,13 +718,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -730,49 +790,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -790,25 +814,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -820,19 +832,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -843,6 +843,30 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -891,21 +915,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -929,15 +938,6 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
       </bottom>
@@ -948,142 +948,142 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1902,9 +1902,7 @@
       <c r="L9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="M9" s="8" t="s">
-        <v>23</v>
-      </c>
+      <c r="M9" s="8"/>
       <c r="N9" s="8" t="s">
         <v>23</v>
       </c>
@@ -1915,7 +1913,7 @@
         <v>18</v>
       </c>
       <c r="Q9" s="8" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" s="4" customFormat="1" spans="1:17">

</xml_diff>